<commit_message>
Merged PR 2186: Merge MahadevProductB to master
I have updated code in ProjectManager.java and ProjectWebServices.java
</commit_message>
<xml_diff>
--- a/src/main/resources/Application_Field_Values.xlsx
+++ b/src/main/resources/Application_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E3D6BC2-EE05-4389-84A7-ADD08AE6C80B}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8BB19A9-465C-4310-BA77-366133DF1336}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="5" xr2:uid="{24C7FA98-EA31-489A-B4B9-70B882520CBB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="5" xr2:uid="{24C7FA98-EA31-489A-B4B9-70B882520CBB}"/>
   </bookViews>
   <sheets>
     <sheet name="CreationPA" sheetId="6" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="79">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -73,18 +73,12 @@
     <t>Automation application Project abstract</t>
   </si>
   <si>
-    <t>Justification__c</t>
-  </si>
-  <si>
     <t>CheckBox</t>
   </si>
   <si>
     <t>Checked</t>
   </si>
   <si>
-    <t>ProjectAbstract__c</t>
-  </si>
-  <si>
     <t>Budget</t>
   </si>
   <si>
@@ -253,29 +247,35 @@
     <t>Non-Construction</t>
   </si>
   <si>
-    <t>PROGRAMINCOME__c</t>
-  </si>
-  <si>
-    <t>ProjectGoal__c</t>
-  </si>
-  <si>
-    <t>ProjectBeneficiaries__c</t>
-  </si>
-  <si>
-    <t>Automation application Project  goal</t>
-  </si>
-  <si>
-    <t>Automation application Project beneficiaries</t>
-  </si>
-  <si>
-    <t>Agreement5__c</t>
+    <t>fieldProjectAbstract__c</t>
+  </si>
+  <si>
+    <t>fieldAcknowledgment4__c</t>
+  </si>
+  <si>
+    <t>fieldJustification__c</t>
+  </si>
+  <si>
+    <t>Proposal</t>
+  </si>
+  <si>
+    <t>fieldApproachMethodology__c</t>
+  </si>
+  <si>
+    <t>Automation Test Description</t>
+  </si>
+  <si>
+    <t>fieldCapacity__c</t>
+  </si>
+  <si>
+    <t>fieldQualifications__c</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -297,6 +297,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF222222"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -320,7 +326,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -330,6 +336,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -646,14 +653,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC0ED488-2B1F-4F16-8235-EEBCD02879E6}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -664,37 +671,37 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
         <v>67</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" s="4" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
         <v>69</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C4" t="s">
         <v>70</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>71</v>
-      </c>
-      <c r="C4" t="s">
-        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -705,13 +712,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA4273BE-F829-4298-BC03-1F37623C37B1}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -722,147 +729,147 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
         <v>36</v>
-      </c>
-      <c r="C2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>38</v>
       </c>
       <c r="C3">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
         <v>39</v>
       </c>
-      <c r="C4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
         <v>40</v>
       </c>
-      <c r="C5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="C7" t="s">
         <v>41</v>
       </c>
-      <c r="C6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" t="s">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
         <v>42</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
         <v>44</v>
       </c>
-      <c r="C8" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
         <v>45</v>
       </c>
-      <c r="C9" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
         <v>46</v>
       </c>
-      <c r="C10" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>4</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="C12" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
         <v>47</v>
       </c>
-      <c r="C11" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>4</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="C13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
         <v>48</v>
       </c>
-      <c r="C12" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>4</v>
-      </c>
-      <c r="B13" t="s">
-        <v>49</v>
-      </c>
-      <c r="C13" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>4</v>
-      </c>
-      <c r="B14" t="s">
-        <v>50</v>
-      </c>
       <c r="C14" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -873,14 +880,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A408404E-903C-4747-8B93-C5CB9A3B0B16}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -891,133 +898,133 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C3">
         <v>200</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C4" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C5">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C7">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C8">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
       <c r="B9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>60</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="B10" t="s">
         <v>61</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>62</v>
-      </c>
-      <c r="B10" t="s">
-        <v>63</v>
       </c>
       <c r="C10">
         <v>1000</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" t="s">
         <v>62</v>
-      </c>
-      <c r="B11" t="s">
-        <v>64</v>
       </c>
       <c r="C11">
         <v>10000</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B12" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C12">
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B13" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C13">
         <v>100000</v>
@@ -1034,13 +1041,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70B87285-F8C8-4985-8D64-B234A73C3C3A}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="37.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1051,7 +1058,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1059,7 +1066,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -1070,13 +1077,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2428A64E-9297-4AA1-BA48-EB8E69A06CF3}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.5546875" customWidth="1"/>
+    <col min="3" max="3" width="23.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1087,23 +1094,23 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C2">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C3" t="s">
         <v>9</v>
@@ -1117,14 +1124,14 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A097844-34E4-4BE1-AA5B-8A6518D2ECB3}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="44.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1135,88 +1142,94 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
       <c r="B3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>74</v>
       </c>
-      <c r="C3" t="s">
+      <c r="B5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C5" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C4" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" t="s">
-        <v>73</v>
-      </c>
-      <c r="C5">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>74</v>
+      </c>
+      <c r="B7" t="s">
         <v>78</v>
       </c>
-      <c r="C6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" t="s">
-        <v>13</v>
-      </c>
       <c r="C7" t="s">
-        <v>33</v>
-      </c>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B8" s="5"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B9" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78E5D97A-D013-4183-BB17-5426A6B81276}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="76.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="76.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1227,125 +1240,125 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
         <v>19</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
         <v>21</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
         <v>23</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="C6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
         <v>25</v>
       </c>
-      <c r="C5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="C7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
         <v>26</v>
       </c>
-      <c r="C6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
         <v>27</v>
       </c>
-      <c r="C7" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
         <v>28</v>
       </c>
-      <c r="C8" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
         <v>29</v>
       </c>
-      <c r="C9" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
         <v>30</v>
       </c>
-      <c r="C10" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>4</v>
-      </c>
-      <c r="B11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>4</v>
-      </c>
-      <c r="B12" t="s">
-        <v>32</v>
-      </c>
       <c r="C12" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -1357,13 +1370,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8676E538-BD44-4E88-B93C-585B884C6D39}">
   <dimension ref="A1:C21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.88671875" customWidth="1"/>
-    <col min="2" max="2" width="11.5546875" customWidth="1"/>
+    <col min="1" max="1" width="10.85546875" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1371,7 +1384,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1379,35 +1392,35 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Merged PR 2384: Merge MahadevProductB to master
application Review.feature- Fixed application review happy path
ProjectManager.java - Added a new step
siteVisit.feature- Fixed scenarios
</commit_message>
<xml_diff>
--- a/src/main/resources/Application_Field_Values.xlsx
+++ b/src/main/resources/Application_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5987853C-84BC-435A-BCCD-A050C6C486EF}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5779D913-74B9-41ED-86A0-6D5653069E19}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{24C7FA98-EA31-489A-B4B9-70B882520CBB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="5" xr2:uid="{24C7FA98-EA31-489A-B4B9-70B882520CBB}"/>
   </bookViews>
   <sheets>
     <sheet name="Editionpre-app" sheetId="6" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="80">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -238,21 +238,9 @@
     <t>ProjectAbstract__c</t>
   </si>
   <si>
-    <t>Acknowledgment4__c</t>
-  </si>
-  <si>
     <t>Justification__c</t>
   </si>
   <si>
-    <t>ApproachMethodology__c</t>
-  </si>
-  <si>
-    <t>Capacity__c</t>
-  </si>
-  <si>
-    <t>Qualifications__c</t>
-  </si>
-  <si>
     <t>ProjectGoal__c</t>
   </si>
   <si>
@@ -266,13 +254,31 @@
   </si>
   <si>
     <t>Agreement5__c</t>
+  </si>
+  <si>
+    <t>fieldAcknowledgment4__c</t>
+  </si>
+  <si>
+    <t>fieldProjectAbstract__c</t>
+  </si>
+  <si>
+    <t>fieldJustification__c</t>
+  </si>
+  <si>
+    <t>fieldApproachMethodology__c</t>
+  </si>
+  <si>
+    <t>fieldCapacity__c</t>
+  </si>
+  <si>
+    <t>fieldQualifications__c</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -287,12 +293,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF222222"/>
-      <name val="Consolas"/>
-      <family val="3"/>
     </font>
     <font>
       <sz val="7"/>
@@ -322,7 +322,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -332,7 +332,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -649,14 +648,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC0ED488-2B1F-4F16-8235-EEBCD02879E6}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -667,7 +666,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -678,45 +677,45 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>74</v>
+      <c r="B3" s="4" t="s">
+        <v>70</v>
       </c>
       <c r="C3" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>73</v>
-      </c>
-      <c r="C4" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>77</v>
       </c>
       <c r="C5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C6" t="s">
         <v>31</v>
@@ -731,13 +730,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA4273BE-F829-4298-BC03-1F37623C37B1}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -748,7 +747,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -759,7 +758,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -770,7 +769,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -781,7 +780,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -792,7 +791,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -803,7 +802,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -814,7 +813,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -825,7 +824,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -836,7 +835,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -847,7 +846,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -858,7 +857,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -869,7 +868,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -880,7 +879,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -899,14 +898,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A408404E-903C-4747-8B93-C5CB9A3B0B16}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -917,7 +916,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -928,7 +927,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -939,7 +938,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -950,7 +949,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -961,7 +960,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -972,7 +971,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -983,7 +982,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -994,7 +993,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -1005,7 +1004,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>60</v>
       </c>
@@ -1016,7 +1015,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>60</v>
       </c>
@@ -1027,7 +1026,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>60</v>
       </c>
@@ -1038,7 +1037,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>60</v>
       </c>
@@ -1060,13 +1059,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70B87285-F8C8-4985-8D64-B234A73C3C3A}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="37.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1077,7 +1076,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1096,13 +1095,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2428A64E-9297-4AA1-BA48-EB8E69A06CF3}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.5546875" customWidth="1"/>
+    <col min="3" max="3" width="23.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1113,7 +1112,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1124,7 +1123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1143,14 +1142,14 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A097844-34E4-4BE1-AA5B-8A6518D2ECB3}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="44.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1161,77 +1160,71 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="C4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>65</v>
       </c>
       <c r="B5" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="C5" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>65</v>
       </c>
       <c r="B6" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="C6" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>65</v>
       </c>
       <c r="B7" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="C7" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B8" s="4"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B9" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1242,13 +1235,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78E5D97A-D013-4183-BB17-5426A6B81276}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="76.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="76.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1259,7 +1252,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1270,7 +1263,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1281,7 +1274,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1292,7 +1285,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1303,7 +1296,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1314,7 +1307,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1325,7 +1318,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1336,7 +1329,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1347,7 +1340,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -1358,7 +1351,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -1369,7 +1362,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1389,13 +1382,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8676E538-BD44-4E88-B93C-585B884C6D39}">
   <dimension ref="A1:C21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.88671875" customWidth="1"/>
-    <col min="2" max="2" width="11.5546875" customWidth="1"/>
+    <col min="1" max="1" width="10.85546875" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1403,7 +1396,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1411,7 +1404,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1419,27 +1412,27 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
fixed application intake WB file
</commit_message>
<xml_diff>
--- a/src/main/resources/Application_Field_Values.xlsx
+++ b/src/main/resources/Application_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10113"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jitendrapisal/rei/govgrants-product-automation/src/main/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7249333F-2162-4D59-A5A5-99B060D44EE3}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09959F57-D600-2E4A-831D-215F6EF1B2DA}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{24C7FA98-EA31-489A-B4B9-70B882520CBB}"/>
+    <workbookView xWindow="0" yWindow="460" windowWidth="23260" windowHeight="12580" activeTab="2" xr2:uid="{24C7FA98-EA31-489A-B4B9-70B882520CBB}"/>
   </bookViews>
   <sheets>
     <sheet name="Editionpre-app" sheetId="6" r:id="rId1"/>
@@ -282,17 +282,17 @@
     <t>Addressline1__c</t>
   </si>
   <si>
-    <t>city__c</t>
-  </si>
-  <si>
     <t>Herndon</t>
+  </si>
+  <si>
+    <t>City__c</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -313,6 +313,12 @@
       <color rgb="FF222222"/>
       <name val="Consolas"/>
       <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF222222"/>
+      <name val="Menlo"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -336,7 +342,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -346,6 +352,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -662,14 +669,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC0ED488-2B1F-4F16-8235-EEBCD02879E6}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="43.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -680,7 +687,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -691,7 +698,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -702,7 +709,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -713,7 +720,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -724,7 +731,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -744,13 +751,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8676E538-BD44-4E88-B93C-585B884C6D39}">
   <dimension ref="A1:C21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.88671875" customWidth="1"/>
-    <col min="2" max="2" width="11.5546875" customWidth="1"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -758,7 +765,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -766,7 +773,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -774,27 +781,27 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>10</v>
       </c>
@@ -813,13 +820,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{766848EE-2835-4541-A2DE-2EBCDE357668}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="44.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -830,7 +837,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -841,7 +848,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -852,7 +859,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>65</v>
       </c>
@@ -863,7 +870,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>65</v>
       </c>
@@ -874,7 +881,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>65</v>
       </c>
@@ -893,13 +900,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D16F34EE-937B-4D9C-AA9F-266997B4D30C}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -910,7 +917,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -921,15 +928,15 @@
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C3" t="s">
         <v>82</v>
-      </c>
-      <c r="C3" t="s">
-        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -941,13 +948,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA4273BE-F829-4298-BC03-1F37623C37B1}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -958,7 +965,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -969,7 +976,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -980,7 +987,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -991,7 +998,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1002,7 +1009,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1013,7 +1020,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1024,7 +1031,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1035,7 +1042,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1046,7 +1053,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -1057,7 +1064,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -1068,7 +1075,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1079,7 +1086,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -1090,7 +1097,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -1109,14 +1116,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A408404E-903C-4747-8B93-C5CB9A3B0B16}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1127,7 +1134,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1138,7 +1145,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -1149,7 +1156,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1160,7 +1167,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -1171,7 +1178,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -1182,7 +1189,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -1193,7 +1200,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -1204,7 +1211,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -1215,7 +1222,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>60</v>
       </c>
@@ -1226,7 +1233,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>60</v>
       </c>
@@ -1237,7 +1244,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>60</v>
       </c>
@@ -1248,7 +1255,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>60</v>
       </c>
@@ -1270,13 +1277,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70B87285-F8C8-4985-8D64-B234A73C3C3A}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="37.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1287,7 +1294,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1306,13 +1313,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2428A64E-9297-4AA1-BA48-EB8E69A06CF3}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.5546875" customWidth="1"/>
+    <col min="3" max="3" width="23.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1323,7 +1330,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1334,7 +1341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1354,13 +1361,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A097844-34E4-4BE1-AA5B-8A6518D2ECB3}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="44.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1371,7 +1378,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1382,7 +1389,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -1393,7 +1400,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -1404,7 +1411,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>65</v>
       </c>
@@ -1415,7 +1422,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>65</v>
       </c>
@@ -1426,7 +1433,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>65</v>
       </c>
@@ -1446,13 +1453,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78E5D97A-D013-4183-BB17-5426A6B81276}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="76.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="76.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1463,7 +1470,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1474,7 +1481,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1485,7 +1492,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1496,7 +1503,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1507,7 +1514,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1518,7 +1525,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1529,7 +1536,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1540,7 +1547,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1551,7 +1558,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -1562,7 +1569,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -1573,7 +1580,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>4</v>
       </c>

</xml_diff>